<commit_message>
Add PDF Name column to latest image assignment workbook
</commit_message>
<xml_diff>
--- a/images/image_assignment_sheet_ignore_first_page.xlsx
+++ b/images/image_assignment_sheet_ignore_first_page.xlsx
@@ -428,15 +428,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,25 +448,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>PDF Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Image Screen Shot url</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Assigned on</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Alt Text</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Long Description</t>
         </is>
@@ -479,13 +485,18 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>124-0047-1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/124-0047-1_2.png</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -495,13 +506,18 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>124-0047-1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/124-0047-1_3.png</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -511,13 +527,18 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>124-0047-1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/124-0047-1_4.png</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -527,13 +548,18 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>124-0047-1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/124-0047-1_5.png</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -543,13 +569,18 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>21-case09</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/21-case09_9.png</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -559,13 +590,18 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>22-case10</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/22-case10_9.png</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -575,13 +611,18 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>24-case12</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/24-case12_7.png</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -591,13 +632,18 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>25-case13</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/25-case13_3.png</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -607,13 +653,18 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>31-case19</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/31-case19_4.png</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -623,13 +674,18 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>31-case19</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/31-case19_5.png</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -639,13 +695,18 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>324-0169-1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0169-1_11.png</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -655,13 +716,18 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>324-0169-1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0169-1_2.png</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -671,13 +737,18 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
+          <t>324-0169-1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0169-1_3.png</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -687,13 +758,18 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>324-0169-1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0169-1_4.png</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -703,13 +779,18 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>324-0169-1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0169-1_7.png</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -719,13 +800,18 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>324-0169-1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0169-1_8.png</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -735,13 +821,18 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
+          <t>324-0321-1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0321-1_10.png</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -751,13 +842,18 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
+          <t>324-0321-1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0321-1_11.png</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -767,13 +863,18 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>324-0321-1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/324-0321-1_2.png</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -783,13 +884,18 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
+          <t>325-0058-1</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0058-1_3.png</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -799,13 +905,18 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
+          <t>325-0058-1</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0058-1_4.png</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -815,13 +926,18 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
+          <t>325-0078-1</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0078-1_2.png</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -831,13 +947,18 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>325-0078-1</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0078-1_3.png</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -847,13 +968,18 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
+          <t>325-0081-1</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0081-1_13.png</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -863,13 +989,18 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>325-0081-1</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0081-1_17.png</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -879,13 +1010,18 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>325-0081-1</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0081-1_18.png</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -895,13 +1031,18 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
+          <t>325-0102-1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0102-1_2.png</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -911,13 +1052,18 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>325-0102-1</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0102-1_6.png</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -927,13 +1073,18 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>325-0102-1</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0102-1_7.png</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -943,13 +1094,18 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
+          <t>325-0102-1</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0102-1_8.png</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -959,13 +1115,18 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
+          <t>325-0102-1</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0102-1_9.png</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -975,13 +1136,18 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t>325-0164-1</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0164-1_2.png</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -991,13 +1157,18 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
+          <t>325-0164-1</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0164-1_5.png</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1007,13 +1178,18 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>325-0164-1</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0164-1_6.png</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1023,13 +1199,18 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>325-0175-1</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0175-1_2.png</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1039,13 +1220,18 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
+          <t>325-0175-1</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0175-1_5.png</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1055,13 +1241,18 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
+          <t>325-0175-1</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/325-0175-1_6.png</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1071,13 +1262,18 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
+          <t>424-0055-1</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/424-0055-1_11.png</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1087,13 +1283,18 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
+          <t>424-0055-1</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/424-0055-1_2.png</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1103,13 +1304,18 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
+          <t>424-0057-1</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/424-0057-1_2.png</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1119,13 +1325,18 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
+          <t>425-0018-1</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/425-0018-1_2.png</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1135,13 +1346,18 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>425-0018-1</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/425-0018-1_9.png</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1151,13 +1367,18 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
+          <t>425-0026-1</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/425-0026-1_9.png</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1167,13 +1388,18 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
+          <t>425-0030-1</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/425-0030-1_12.png</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1183,13 +1409,18 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
+          <t>425-0030-1</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/425-0030-1_13.png</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1199,13 +1430,18 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
+          <t>525-0060-1</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/525-0060-1_2.png</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1215,13 +1451,18 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>525-0060-1</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/525-0060-1_7.png</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1231,13 +1472,18 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
+          <t>525-0060-1</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/525-0060-1_8.png</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="2" t="inlineStr"/>
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1247,13 +1493,18 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>624-0046-1</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/624-0046-1_11.png</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1263,13 +1514,18 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
+          <t>624-0046-1</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/624-0046-1_2.png</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="2" t="inlineStr"/>
       <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1279,13 +1535,18 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
+          <t>624-0046-1</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/624-0046-1_4.png</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1295,13 +1556,18 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
+          <t>624-0046-1</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/624-0046-1_5.png</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="2" t="inlineStr"/>
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1311,13 +1577,18 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
+          <t>624-0046-1</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/624-0046-1_7.png</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1327,13 +1598,18 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
+          <t>624-0046-1</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/624-0046-1_9.png</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="inlineStr"/>
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1343,13 +1619,18 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
+          <t>625-0007-1</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0007-1_11.png</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1359,13 +1640,18 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
+          <t>625-0007-1</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0007-1_13.png</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="2" t="inlineStr"/>
       <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1375,13 +1661,18 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
+          <t>625-0007-1</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0007-1_2.png</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1391,13 +1682,18 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
+          <t>625-0010-5</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0010-5_14.png</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="inlineStr"/>
       <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1407,13 +1703,18 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
+          <t>625-0010-5</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0010-5_16.png</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1423,13 +1724,18 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
+          <t>625-0011-1</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0011-1_2.png</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="inlineStr"/>
       <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1439,13 +1745,18 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
+          <t>625-0011-1</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0011-1_3.png</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1455,13 +1766,18 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
+          <t>625-0011-1</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0011-1_5.png</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="inlineStr"/>
       <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1471,13 +1787,18 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
+          <t>625-0011-1</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0011-1_6.png</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1487,13 +1808,18 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_11.png</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="inlineStr"/>
       <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1503,13 +1829,18 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_12.png</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1519,13 +1850,18 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_13.png</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1535,13 +1871,18 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_14.png</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1551,13 +1892,18 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_15.png</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="2" t="inlineStr"/>
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1567,13 +1913,18 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_16.png</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1583,13 +1934,18 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_18.png</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="2" t="inlineStr"/>
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1599,13 +1955,18 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_3.png</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -1615,13 +1976,18 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_5.png</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="2" t="inlineStr"/>
       <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1631,13 +1997,18 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_7.png</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1647,13 +2018,18 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
+          <t>625-0013-5</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/625-0013-5_8.png</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="2" t="inlineStr"/>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -1663,13 +2039,18 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
+          <t>825-0018-1</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0018-1_2.png</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -1679,13 +2060,18 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
+          <t>825-0022-1</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0022-1_12.png</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="2" t="inlineStr"/>
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -1695,13 +2081,18 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
+          <t>825-0022-1</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0022-1_2.png</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="inlineStr"/>
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -1711,13 +2102,18 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
+          <t>825-0022-1</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0022-1_4.png</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr"/>
       <c r="D79" s="2" t="inlineStr"/>
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1727,13 +2123,18 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
+          <t>825-0022-1</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0022-1_6.png</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -1743,13 +2144,18 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
+          <t>825-0022-1</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0022-1_8.png</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr"/>
       <c r="D81" s="2" t="inlineStr"/>
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1759,13 +2165,18 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
+          <t>825-0022-1</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0022-1_9.png</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr"/>
       <c r="D82" s="2" t="inlineStr"/>
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1775,13 +2186,18 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
+          <t>825-0024-1</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0024-1_11.png</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr"/>
       <c r="D83" s="2" t="inlineStr"/>
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1791,13 +2207,18 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
+          <t>825-0024-1</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/825-0024-1_12.png</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr"/>
       <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -1807,13 +2228,18 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
+          <t>924-0022-1</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/924-0022-1_11.png</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr"/>
       <c r="D85" s="2" t="inlineStr"/>
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1823,13 +2249,18 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
+          <t>924-0022-1</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/924-0022-1_2.png</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="2" t="inlineStr"/>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -1839,13 +2270,18 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>924-0022-1</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/924-0022-1_4.png</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="2" t="inlineStr"/>
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1855,13 +2291,18 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
+          <t>924-0022-1</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/924-0022-1_6.png</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="2" t="inlineStr"/>
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -1871,13 +2312,18 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
+          <t>924-0022-1</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/924-0022-1_7.png</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="2" t="inlineStr"/>
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1887,13 +2333,18 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
+          <t>925-0004-1</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0004-1_11.png</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr"/>
       <c r="D90" s="2" t="inlineStr"/>
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1903,13 +2354,18 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
+          <t>925-0004-1</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0004-1_12.png</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr"/>
       <c r="D91" s="2" t="inlineStr"/>
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1919,13 +2375,18 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>925-0004-1</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0004-1_13.png</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="2" t="inlineStr"/>
       <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1935,13 +2396,18 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
+          <t>925-0004-1</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0004-1_2.png</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="2" t="inlineStr"/>
       <c r="E93" s="2" t="inlineStr"/>
       <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -1951,13 +2417,18 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
+          <t>925-0005-1</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0005-1_10.png</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr"/>
       <c r="D94" s="2" t="inlineStr"/>
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -1967,13 +2438,18 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
+          <t>925-0005-1</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0005-1_12.png</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr"/>
       <c r="D95" s="2" t="inlineStr"/>
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1983,13 +2459,18 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
+          <t>925-0005-1</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0005-1_13.png</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr"/>
       <c r="D96" s="2" t="inlineStr"/>
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1999,13 +2480,18 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
+          <t>925-0005-1</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0005-1_2.png</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr"/>
       <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2015,13 +2501,18 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
+          <t>925-0010-1</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0010-1_2.png</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr"/>
       <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2031,13 +2522,18 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
+          <t>925-0010-1</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0010-1_9.png</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr"/>
       <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2047,13 +2543,18 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
+          <t>925-0019-1</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/925-0019-1_2.png</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr"/>
       <c r="D100" s="2" t="inlineStr"/>
       <c r="E100" s="2" t="inlineStr"/>
       <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2063,13 +2564,18 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
+          <t>KE1302</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/KE1302_10.png</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr"/>
       <c r="D101" s="2" t="inlineStr"/>
       <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2079,13 +2585,18 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
+          <t>KE1302</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/KE1302_3.png</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr"/>
       <c r="D102" s="2" t="inlineStr"/>
       <c r="E102" s="2" t="inlineStr"/>
       <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2095,13 +2606,18 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
+          <t>KE1302</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/KE1302_8.png</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr"/>
       <c r="D103" s="2" t="inlineStr"/>
       <c r="E103" s="2" t="inlineStr"/>
       <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -2111,13 +2627,18 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
+          <t>KE1302</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
           <t>https://raw.githubusercontent.com/dakshsolution/daksh-31d6cfe0/main/images/KE1302_9.png</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr"/>
       <c r="D104" s="2" t="inlineStr"/>
       <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>